<commit_message>
feat(fichas): GRA agrega grafico de recta de flujo (semi-log) del Limite Liquido, completando el requisito grafico del protocolo Atterberg
</commit_message>
<xml_diff>
--- a/Proyectos Modelo/Proyecto_Carretera/GRA_GranulometriaAtterberg.xlsx
+++ b/Proyectos Modelo/Proyecto_Carretera/GRA_GranulometriaAtterberg.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -770,13 +770,13 @@
         <v>18</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>Recta de flujo (semi-log)</v>
       </c>
       <c r="E19" t="str">
-        <v>col-[A][Rollo 1] // col-[B][Rollo 2]</v>
+        <v>numerico-gr5[x:#14A:#14C|y:#15A:#15C|alto:55|t:Recta de Flujo — Límite Líquido|xt:N° de golpes|yt:Humedad (%)|ly:Puntos de ensayo]</v>
       </c>
       <c r="F19" t="str">
-        <v>Límite Plástico e Índice de Plasticidad</v>
+        <v>Límite Líquido (copa de Casagrande)</v>
       </c>
     </row>
     <row r="20">
@@ -790,10 +790,10 @@
         <v>19</v>
       </c>
       <c r="D20" t="str">
-        <v>Contenido de humedad (%)</v>
+        <v/>
       </c>
       <c r="E20" t="str">
-        <v>numerico-[10:40]:dec[1]:ej[17.6] // numerico-[10:40]:dec[1]:ej[17.4]</v>
+        <v>col-[A][Rollo 1] // col-[B][Rollo 2]</v>
       </c>
       <c r="F20" t="str">
         <v>Límite Plástico e Índice de Plasticidad</v>
@@ -810,10 +810,10 @@
         <v>20</v>
       </c>
       <c r="D21" t="str">
-        <v>Límite Plástico — LP (%)</v>
+        <v>Contenido de humedad (%)</v>
       </c>
       <c r="E21" t="str">
-        <v>numerico-fx[PROMEDIO(#19A:#19B)]:dec[1]</v>
+        <v>numerico-[10:40]:dec[1]:ej[17.6] // numerico-[10:40]:dec[1]:ej[17.4]</v>
       </c>
       <c r="F21" t="str">
         <v>Límite Plástico e Índice de Plasticidad</v>
@@ -830,10 +830,10 @@
         <v>21</v>
       </c>
       <c r="D22" t="str">
-        <v>Índice de Plasticidad — IP (%)</v>
+        <v>Límite Plástico — LP (%)</v>
       </c>
       <c r="E22" t="str">
-        <v>numerico-fx[#17A-#20A]:dec[1]</v>
+        <v>numerico-fx[PROMEDIO(#20A:#20B)]:dec[1]</v>
       </c>
       <c r="F22" t="str">
         <v>Límite Plástico e Índice de Plasticidad</v>
@@ -850,13 +850,13 @@
         <v>22</v>
       </c>
       <c r="D23" t="str">
-        <v>% de finos (pasa N° 200)</v>
+        <v>Índice de Plasticidad — IP (%)</v>
       </c>
       <c r="E23" t="str">
-        <v>numerico-fx[#10E]:dec[1]</v>
+        <v>numerico-fx[#17A-#21A]:dec[1]</v>
       </c>
       <c r="F23" t="str">
-        <v>Evaluación de cumplimiento</v>
+        <v>Límite Plástico e Índice de Plasticidad</v>
       </c>
     </row>
     <row r="24">
@@ -870,10 +870,10 @@
         <v>23</v>
       </c>
       <c r="D24" t="str">
-        <v>LL máximo por la capa (%)</v>
+        <v>% de finos (pasa N° 200)</v>
       </c>
       <c r="E24" t="str">
-        <v>numerico-fx[BUSCAR(capas_pavimento, #2A, LLmax)]:dec[1]</v>
+        <v>numerico-fx[#10E]:dec[1]</v>
       </c>
       <c r="F24" t="str">
         <v>Evaluación de cumplimiento</v>
@@ -890,10 +890,10 @@
         <v>24</v>
       </c>
       <c r="D25" t="str">
-        <v>IP máximo por la capa (%)</v>
+        <v>LL máximo por la capa (%)</v>
       </c>
       <c r="E25" t="str">
-        <v>numerico-fx[BUSCAR(capas_pavimento, #2A, IPmax)]:dec[1]</v>
+        <v>numerico-fx[BUSCAR(capas_pavimento, #2A, LLmax)]:dec[1]</v>
       </c>
       <c r="F25" t="str">
         <v>Evaluación de cumplimiento</v>
@@ -910,10 +910,10 @@
         <v>25</v>
       </c>
       <c r="D26" t="str">
-        <v>¿Cumple Límite Líquido? (1=Sí, 0=No)</v>
+        <v>IP máximo por la capa (%)</v>
       </c>
       <c r="E26" t="str">
-        <v>numerico-fx[SI(#17A&lt;=#23A,1,0)]:dec[0]</v>
+        <v>numerico-fx[BUSCAR(capas_pavimento, #2A, IPmax)]:dec[1]</v>
       </c>
       <c r="F26" t="str">
         <v>Evaluación de cumplimiento</v>
@@ -930,10 +930,10 @@
         <v>26</v>
       </c>
       <c r="D27" t="str">
-        <v>¿Cumple Índice de Plasticidad? (1=Sí, 0=No)</v>
+        <v>¿Cumple Límite Líquido? (1=Sí, 0=No)</v>
       </c>
       <c r="E27" t="str">
-        <v>numerico-fx[SI(#21A&lt;=#24A,1,0)]:dec[0]</v>
+        <v>numerico-fx[SI(#17A&lt;=#24A,1,0)]:dec[0]</v>
       </c>
       <c r="F27" t="str">
         <v>Evaluación de cumplimiento</v>
@@ -950,18 +950,38 @@
         <v>27</v>
       </c>
       <c r="D28" t="str">
-        <v>Dictamen final (1=CONFORME, 0=NO CONFORME)</v>
+        <v>¿Cumple Índice de Plasticidad? (1=Sí, 0=No)</v>
       </c>
       <c r="E28" t="str">
-        <v>numerico-fx[SI(Y(#25A&gt;=1,#26A&gt;=1),1,0)]:dec[0]</v>
+        <v>numerico-fx[SI(#22A&lt;=#25A,1,0)]:dec[0]</v>
       </c>
       <c r="F28" t="str">
         <v>Evaluación de cumplimiento</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>GRA</v>
+      </c>
+      <c r="B29" t="str">
+        <v>GRANULOMETRIA Y ATTERBERG</v>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Dictamen final (1=CONFORME, 0=NO CONFORME)</v>
+      </c>
+      <c r="E29" t="str">
+        <v>numerico-fx[SI(Y(#26A&gt;=1,#27A&gt;=1),1,0)]:dec[0]</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Evaluación de cumplimiento</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>